<commit_message>
agrega pruebas de proveedores y responsividad, y revisión del diseño adaptable
- pruebas de CarritoProvider (con temporizadores simulados),
DatosProvider y useTitulo
- pruebas de las clases responsivas de Bootstrap (menú, rejilla y
tablas)
- docs/responsividad.md: revisión de 35 rutas a 375, 768 y 1280
px, sin desbordes
- cobertura: 99,32 % sentencias, 94,58 % ramas, 99,80 %
funciones y 99,51 % líneas (760 pruebas en 85 archivos)
- actualiza cobertura-testing.md, README, paridad-react.md
y la cifra de RNF-09 en el ERS y la planilla de requerimientos
</commit_message>
<xml_diff>
--- a/Planilla de Requerimientos - Ensambla.me.xlsx
+++ b/Planilla de Requerimientos - Ensambla.me.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requerimiento Inicial" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Requerimiento Inicial'!$A$1:$H$24</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Requerimiento Inicial'!$A$1:$H$36</definedName>
   </definedNames>
   <calcPr calcId="152511" fullCalcOnLoad="1"/>
 </workbook>
@@ -623,7 +623,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H24"/>
+  <dimension ref="A1:H36"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
   <cols>
     <col width="8.109375" customWidth="1" min="1" max="1"/>
@@ -631,7 +631,7 @@
     <col width="25.6640625" customWidth="1" min="3" max="4"/>
     <col width="25.5" customWidth="1" min="4" max="4"/>
     <col width="25.5546875" customWidth="1" min="5" max="5"/>
-    <col width="66.109375" customWidth="1" min="6" max="6"/>
+    <col width="80" customWidth="1" min="6" max="6"/>
     <col width="80" customWidth="1" min="7" max="7"/>
     <col width="15.88671875" customWidth="1" min="8" max="8"/>
   </cols>
@@ -679,7 +679,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="259" customHeight="1">
+    <row r="2" ht="293" customHeight="1">
       <c r="A2" s="12" t="inlineStr">
         <is>
           <t>RF-01</t>
@@ -718,7 +718,7 @@
 4. Una contraseña de menos de 4 o más de 10 caracteres se rechaza con su error.
 5. Cuando se cambia la región seleccionada, el select de comuna se recarga únicamente con las comunas de esa región.
 6. Los valores que superan los máximos definidos (nombre &gt; 50, apellidos &gt; 100, correo &gt; 100, dirección &gt; 300 caracteres) no pueden ingresarse o muestran el error correspondiente.
-7. Cuando se envía un formulario completo y válido, el usuario se agrega al arreglo de usuarios y se muestra un mensaje de confirmación.
+7. Cuando se envía un formulario completo y válido, el usuario se agrega a los datos de usuarios con el tipo Cliente y se muestra un mensaje de confirmación; un RUN o un correo ya registrados se rechazan.
 8. El campo de correo ofrece los dominios permitidos como sugerencia seleccionable (datalist), de modo que puedan completarse sin escribirlos.</t>
         </is>
       </c>
@@ -728,7 +728,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="124" customHeight="1">
+    <row r="3" ht="158" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
           <t>RF-02</t>
@@ -761,7 +761,7 @@
       </c>
       <c r="G3" s="12" t="inlineStr">
         <is>
-          <t>1. Cuando el correo y la contraseña coinciden con un usuario registrado, la sesión se inicia y se habilitan las funcionalidades de su rol: el rol Cliente llega a la tienda pública; el rol Administrador, al panel de gestión con sus mantenedores (RF-10 y RF-11); el rol Administrador logístico, a productos y órdenes en solo lectura (RF-12).
+          <t>1. Cuando el correo y la contraseña coinciden con un usuario registrado, la sesión se inicia y el usuario llega a la vista que había pedido, si esa ruta es del mismo sitio, o, si no la había, a la que corresponde a su rol: el rol Cliente, la tienda pública; el rol Administrador, el panel de gestión con sus mantenedores (RF-10, RF-11 y RF-25); el rol Administrador logístico, los productos y órdenes en solo lectura (RF-12).
 2. Un correo de dominio no permitido o una contraseña de menos de 4 o más de 10 caracteres se rechazan con su error y el formulario no se envía.
 3. Unas credenciales que no coinciden con ningún usuario producen un mensaje genérico ("correo o contraseña incorrectos"), sin revelar cuál de los dos falló.</t>
         </is>
@@ -772,7 +772,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="109" customHeight="1">
+    <row r="4" ht="113" customHeight="1">
       <c r="A4" s="12" t="inlineStr">
         <is>
           <t>RF-03</t>
@@ -800,14 +800,14 @@
       </c>
       <c r="F4" s="12" t="inlineStr">
         <is>
-          <t>El cliente debe poder consultar el catálogo de productos y ver de cada uno su imagen, su nombre y su precio. El listado debe obtenerse de los datos de productos y no del marcado de la vista, de modo que agregar un producto a los datos baste para que aparezca. Las vistas que presentan el catálogo y la disposición de sus elementos se especifican en 3.1.1.</t>
+          <t>El cliente debe poder consultar el catálogo de productos y ver de cada uno su imagen, su nombre, su categoría y su precio vigente (RF-18). El listado debe obtenerse de los datos de productos y no del marcado de la vista, de modo que agregar un producto a los datos baste para que aparezca. La búsqueda y los filtros del catálogo se especifican en RF-17, y las vistas que presentan el catálogo y la disposición de sus elementos, en 3.1.1.</t>
         </is>
       </c>
       <c r="G4" s="12" t="inlineStr">
         <is>
-          <t>1. Al cargar una vista de catálogo se renderiza una tarjeta por cada producto con su imagen, nombre y precio; al agregar un elemento a los datos y recargar la página, la nueva tarjeta aparece sin haber modificado el HTML, lo que demuestra que el listado se genera dinámicamente.
+          <t>1. Al cargar una vista de catálogo se renderiza una tarjeta por cada producto con su imagen, nombre, categoría y precio; al agregar un producto a los datos, la nueva tarjeta aparece sin haber modificado los componentes, lo que demuestra que el listado se genera dinámicamente.
 2. Los precios se muestran formateados como moneda (pesos chilenos).
-3. Con el arreglo de productos vacío, la vista muestra un mensaje de "no hay productos disponibles" en lugar de un área en blanco.</t>
+3. Sin productos, la vista muestra un aviso de "no hay productos disponibles" en lugar de un área en blanco.</t>
         </is>
       </c>
       <c r="H4" s="12" t="inlineStr">
@@ -816,7 +816,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="139" customHeight="1">
+    <row r="5" ht="158" customHeight="1">
       <c r="A5" s="12" t="inlineStr">
         <is>
           <t>RF-04</t>
@@ -850,8 +850,8 @@
       <c r="G5" s="12" t="inlineStr">
         <is>
           <t>1. Al hacer clic sobre un producto del listado se navega al detalle de ese producto y no de otro.
-2. El detalle muestra imagen, nombre, precio, descripción y categoría del producto seleccionado, e incluye un botón "Añadir al carrito" operativo (RF-05).
-3. Un código de producto que no existe en el arreglo produce un mensaje de producto no encontrado, en lugar de una vista vacía o un error de JavaScript.
+2. El detalle muestra imagen, nombre, precio vigente, descripción, categoría y stock del producto seleccionado, e incluye un botón "Añadir al carrito" operativo (RF-05).
+3. Un código de producto que no existe en los datos produce un mensaje de producto no encontrado, en lugar de una vista vacía o un error de JavaScript.
 4. Dado un producto que define el campo video, su detalle lo muestra embebido y reproducible sin salir del sitio; si no lo define, la vista se muestra completa y sin contenedores vacíos.</t>
         </is>
       </c>
@@ -861,7 +861,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="169" customHeight="1">
+    <row r="6" ht="173" customHeight="1">
       <c r="A6" s="12" t="inlineStr">
         <is>
           <t>RF-05</t>
@@ -907,7 +907,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="184" customHeight="1">
+    <row r="7" ht="233" customHeight="1">
       <c r="A7" s="12" t="inlineStr">
         <is>
           <t>RF-06</t>
@@ -935,16 +935,16 @@
       </c>
       <c r="F7" s="12" t="inlineStr">
         <is>
-          <t>El cliente debe poder visualizar el contenido del carrito de compras, eliminar un producto del carrito, modificar la cantidad de un ítem y ver el total calculado a partir de los precios y las cantidades. El contenido del carrito debe conservarse entre sesiones del navegador (ver 3.1.3).</t>
+          <t>El cliente debe poder visualizar el contenido del carrito de compras, eliminar un producto del carrito, modificar la cantidad de un ítem, ver el total calculado a partir de los precios vigentes y las cantidades, y continuar al pago (RF-20). El contenido del carrito debe conservarse entre sesiones del navegador (ver 3.1.3).</t>
         </is>
       </c>
       <c r="G7" s="12" t="inlineStr">
         <is>
           <t>1. Cada línea del carrito muestra imagen, nombre, precio unitario, cantidad y subtotal.
 2. Al eliminar un ítem, este desaparece del listado y el total se recalcula sin recargar la página.
-3. Al modificar la cantidad de un ítem se recalculan su subtotal y el total, que corresponde exactamente a la suma de precio unitario por cantidad de todas las líneas; no se permite una cantidad menor que 1 ni una que, sumada a las demás líneas del mismo producto, supere su stock: una cantidad mayor se ajusta al máximo permitido y se informa con un mensaje.
+3. Al modificar la cantidad de un ítem se recalculan su subtotal y el total, que corresponde exactamente a la suma de precio vigente por cantidad de todas las líneas; no se permite una cantidad menor que 1 ni una que, sumada a las demás líneas del mismo producto, supere su stock: una cantidad mayor se ajusta al máximo permitido y se informa con un mensaje.
 4. Dado un carrito con productos, al recargar la página o cerrar y reabrir el navegador el carrito conserva su contenido (persistencia en localStorage); si desde entonces el stock de un producto bajó, su cantidad se ajusta al stock vigente y la línea sin unidades disponibles se quita.
-5. Con el carrito vacío se muestra un mensaje indicándolo y el total es 0.</t>
+5. Con el carrito vacío se muestra un mensaje indicándolo, el total es 0 y la acción de pagar queda deshabilitada.</t>
         </is>
       </c>
       <c r="H7" s="12" t="inlineStr">
@@ -953,7 +953,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="229" customHeight="1">
+    <row r="8" ht="263" customHeight="1">
       <c r="A8" s="12" t="inlineStr">
         <is>
           <t>RF-07</t>
@@ -1001,7 +1001,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="124" customHeight="1">
+    <row r="9" ht="128" customHeight="1">
       <c r="A9" s="12" t="inlineStr">
         <is>
           <t>RF-08</t>
@@ -1046,7 +1046,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="64" customHeight="1">
+    <row r="10" ht="68" customHeight="1">
       <c r="A10" s="12" t="inlineStr">
         <is>
           <t>RF-09</t>
@@ -1089,7 +1089,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="199" customHeight="1">
+    <row r="11" ht="233" customHeight="1">
       <c r="A11" s="12" t="inlineStr">
         <is>
           <t>RF-10</t>
@@ -1117,17 +1117,17 @@
       </c>
       <c r="F11" s="12" t="inlineStr">
         <is>
-          <t>El administrador debe poder listar todos los productos, crear un nuevo producto y editar uno existente, ingresando: código de producto (SKU) (requerido, texto, mín. 3 caracteres, sin límite superior), nombre (requerido, máx. 100), descripción (opcional, máx. 500), precio (requerido, mín. 0 —un valor 0 se considera un producto gratuito—, sin límite superior, admite decimales), stock (requerido, mín. 0, sin límite superior, solo enteros), stock crítico (opcional, mín. 0, solo enteros, muestra alerta cuando el stock sea igual o inferior a este valor), categoría (requerida, escogida entre las categorías del catálogo), imagen (opcional) y video (opcional, URL del video que se muestra en el detalle del producto, ver RF-04).</t>
+          <t>El administrador debe poder listar todos los productos, buscarlos por código, nombre o categoría, crear un nuevo producto, editar uno existente y eliminarlo, ingresando: código de producto (SKU) (requerido, texto, mín. 3 caracteres, único, sin límite superior), nombre (requerido, máx. 100), descripción (opcional, máx. 500), precio (requerido, mín. 0 —un valor 0 se considera un producto gratuito—, sin límite superior, admite decimales), descuento (opcional, entero de 0 a 90, porcentaje que se descuenta del precio de lista; vacío o 0 significa sin oferta, ver RF-18), stock (requerido, mín. 0, sin límite superior, solo enteros), stock crítico (opcional, mín. 0, solo enteros, muestra alerta cuando el stock sea igual o inferior a este valor), categoría (requerida, escogida entre las categorías del catálogo), imagen (opcional) y video (opcional, URL del video que se muestra en el detalle del producto, ver RF-04).</t>
         </is>
       </c>
       <c r="G11" s="12" t="inlineStr">
         <is>
-          <t>1. La vista de listado muestra todos los productos con las acciones de crear y editar disponibles: al crear un producto con un formulario válido este aparece en el listado, y al editar uno existente los cambios se reflejan en él.
-2. Se rechazan con su error un código de menos de 3 caracteres, un precio negativo y un stock negativo o con decimales; el precio admite decimales y un precio 0 se acepta como producto gratuito.
+          <t>1. La vista de listado muestra todos los productos con las acciones de crear, editar y eliminar y una búsqueda por código, nombre o categoría: al crear un producto con un formulario válido este aparece en el listado, y al editar uno existente los cambios se reflejan en él.
+2. Se rechazan con su error un código de menos de 3 caracteres o repetido, un precio negativo, un descuento fuera de 0 a 90 o con decimales, y un stock negativo o con decimales; el precio admite decimales y un precio 0 se acepta como producto gratuito.
 3. Una categoría sin seleccionar impide el envío del formulario, por ser un campo requerido.
 4. Un producto cuyo stock es igual o inferior a su stock crítico muestra una alerta visible de bajo inventario en el listado.
 5. Cuando se guarda una URL en el campo video, el valor se conserva y el detalle del producto lo muestra embebido; dejarlo vacío no impide guardar.
-6. La vista no ofrece la acción Eliminar, que queda fuera del alcance de esta entrega (ver 1.3 y 2.6).</t>
+6. Eliminar un producto pide confirmación; las órdenes que lo incluían conservan su detalle y el carrito descarta la línea.</t>
         </is>
       </c>
       <c r="H11" s="12" t="inlineStr">
@@ -1136,7 +1136,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="169" customHeight="1">
+    <row r="12" ht="203" customHeight="1">
       <c r="A12" s="12" t="inlineStr">
         <is>
           <t>RF-11</t>
@@ -1164,16 +1164,17 @@
       </c>
       <c r="F12" s="12" t="inlineStr">
         <is>
-          <t>El administrador debe poder listar todos los usuarios, crear un nuevo usuario y editar uno existente, con las mismas reglas de campos que RF-01 (incluidos RUN y contraseña), más un campo adicional de tipo de usuario (requerido: Administrador, Cliente o Administrador logístico), que solo puede asignarse desde este mantenedor y no en el registro público (RF-01).</t>
+          <t>El administrador debe poder listar todos los usuarios, buscarlos, crear un nuevo usuario, editar uno existente y eliminarlo, con las mismas reglas de campos que RF-01 (incluidos RUN y contraseña), más un campo adicional de tipo de usuario (requerido: Administrador, Cliente o Administrador logístico), que solo puede asignarse desde este mantenedor y no en el registro público (RF-01). La ficha de cada usuario muestra sus datos, sin la contraseña, y su historial de compras.</t>
         </is>
       </c>
       <c r="G12" s="12" t="inlineStr">
         <is>
-          <t>1. La vista de listado muestra todos los usuarios con las acciones de crear y editar disponibles: al crear un usuario con un formulario válido este aparece en el listado, y al editar uno existente los cambios se reflejan en él.
-2. El formulario de crear o editar usuario aplica las mismas validaciones de RF-01, incluidas las de RUN y contraseña.
+          <t>1. La vista de listado muestra todos los usuarios con las acciones de buscar, crear, editar y eliminar disponibles: al crear un usuario con un formulario válido este aparece en el listado, y al editar uno existente los cambios se reflejan en él.
+2. El formulario de crear o editar usuario aplica las mismas validaciones de RF-01, incluidas las de RUN y contraseña; un RUN o un correo repetidos se rechazan.
 3. El select de tipo de usuario ofrece exactamente las opciones Administrador, Cliente y Administrador logístico, y no aparece en el registro público (RF-01).
 4. Creado un usuario con un rol determinado, al iniciar sesión accede únicamente a lo que su rol permite (RF-02, RF-12).
-5. La vista no ofrece la acción Eliminar, que queda fuera del alcance de esta entrega (ver 1.3 y 2.6).</t>
+5. La ficha del usuario muestra sus datos, sin la contraseña, y su historial de compras con un enlace a la boleta de cada una (RF-24).
+6. Eliminar un usuario pide confirmación y se rechaza si es la cuenta de la sesión actual o si tiene órdenes a su nombre.</t>
         </is>
       </c>
       <c r="H12" s="12" t="inlineStr">
@@ -1182,7 +1183,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="64" customHeight="1">
+    <row r="13" ht="98" customHeight="1">
       <c r="A13" s="12" t="inlineStr">
         <is>
           <t>RF-12</t>
@@ -1190,7 +1191,7 @@
       </c>
       <c r="B13" s="12" t="inlineStr">
         <is>
-          <t>Visualizar productos y órdenes (rol Administrador logístico)</t>
+          <t>Visualizar productos, productos críticos y órdenes (rol Administrador logístico)</t>
         </is>
       </c>
       <c r="C13" s="12" t="inlineStr">
@@ -1210,13 +1211,14 @@
       </c>
       <c r="F13" s="12" t="inlineStr">
         <is>
-          <t>El administrador logístico debe poder visualizar el listado y detalle de productos, y el listado y detalle de órdenes, en modo de solo lectura. La restricción de acceso al resto de las funcionalidades administrativas se especifica en 3.3.2.</t>
+          <t>El administrador logístico debe poder visualizar el listado de productos, los productos críticos (RF-26) y el listado y detalle de órdenes, en modo de solo lectura, y gestionar su propio perfil (RF-23). La restricción de acceso al resto de las funcionalidades administrativas se especifica en 3.3.2.</t>
         </is>
       </c>
       <c r="G13" s="12" t="inlineStr">
         <is>
           <t>1. El listado de productos se muestra en modo lectura, sin botones de crear, editar ni eliminar.
-2. Cada orden del listado muestra cliente, fecha, productos y total, y su detalle también se presenta en modo lectura.</t>
+2. Cada orden del listado muestra cliente, fecha, productos y total; el listado se puede buscar por número, cliente, correo o producto, y el detalle de cada orden es su boleta, en modo lectura.
+3. El rol puede abrir los productos críticos (RF-26) y su propio perfil (RF-23).</t>
         </is>
       </c>
       <c r="H13" s="12" t="inlineStr">
@@ -1225,7 +1227,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="94" customHeight="1">
+    <row r="14" ht="98" customHeight="1">
       <c r="A14" s="12" t="inlineStr">
         <is>
           <t>RF-13</t>
@@ -1269,7 +1271,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="79" customHeight="1">
+    <row r="15" ht="143" customHeight="1">
       <c r="A15" s="12" t="inlineStr">
         <is>
           <t>RF-14</t>
@@ -1297,14 +1299,15 @@
       </c>
       <c r="F15" s="12" t="inlineStr">
         <is>
-          <t>El cliente debe poder desplazarse entre todas las vistas públicas del sitio —inicio, productos, blogs, nosotros y contacto— y conocer en todo momento la cantidad de ítems que contiene su carrito de compras. La disposición de los elementos de navegación se especifica en 3.1.1 y su resolución desde archivos compartidos, en 3.3.5.</t>
+          <t>El cliente debe poder desplazarse entre todas las vistas públicas del sitio —inicio, productos, categorías, ofertas, armado, blogs, nosotros y contacto— y conocer en todo momento la cantidad de ítems que contiene su carrito de compras. La disposición de los elementos de navegación se especifica en 3.1.1 y su resolución desde componentes compartidos, en 3.3.5.</t>
         </is>
       </c>
       <c r="G15" s="12" t="inlineStr">
         <is>
-          <t>1. Cada enlace del menú de navegación conduce a su vista, y el logo de la tienda, a la página de inicio.
+          <t>1. Cada enlace del menú de navegación (Inicio, Productos, Categorías, Ofertas, Armar mi PC, Blogs, Nosotros y Contacto) conduce a su vista, y el logo de la tienda, a la página de inicio.
 2. El acceso al carrito muestra la cantidad de ítems que este contiene y se actualiza al agregar o eliminar productos.
-3. Cada acceso de la barra lateral de categorías navega al listado de productos.</t>
+3. Cada acceso de la barra lateral de categorías navega al listado de productos de esa categoría.
+4. La caja de búsqueda del menú conduce al catálogo con el texto como filtro (RF-17).</t>
         </is>
       </c>
       <c r="H15" s="12" t="inlineStr">
@@ -1313,7 +1316,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="49" customHeight="1">
+    <row r="16" ht="53" customHeight="1">
       <c r="A16" s="12" t="inlineStr">
         <is>
           <t>RF-15</t>
@@ -1355,382 +1358,926 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="109" customHeight="1">
+    <row r="17" ht="188" customHeight="1">
       <c r="A17" s="12" t="inlineStr">
         <is>
+          <t>RF-17</t>
+        </is>
+      </c>
+      <c r="B17" s="12" t="inlineStr">
+        <is>
+          <t>Buscar y filtrar el catálogo</t>
+        </is>
+      </c>
+      <c r="C17" s="12" t="inlineStr">
+        <is>
+          <t>Funcional</t>
+        </is>
+      </c>
+      <c r="D17" s="12" t="inlineStr">
+        <is>
+          <t>Funcional de usuario</t>
+        </is>
+      </c>
+      <c r="E17" s="12" t="inlineStr">
+        <is>
+          <t>Cliente</t>
+        </is>
+      </c>
+      <c r="F17" s="12" t="inlineStr">
+        <is>
+          <t>El cliente debe poder buscar productos por texto, filtrarlos por categoría, rango de precio, ofertas y disponibilidad, y ordenarlos, de modo que encuentre lo que busca sin recorrer todo el catálogo. Los criterios deben quedar en la dirección de la vista para poder compartirla y volver a ella.</t>
+        </is>
+      </c>
+      <c r="G17" s="12" t="inlineStr">
+        <is>
+          <t>1. La búsqueda ignora mayúsculas y tildes y exige que cada palabra aparezca en el nombre, el código, la descripción o la categoría del producto.
+2. Se puede filtrar por categoría, por precio mínimo y máximo (sobre el precio vigente), solo ofertas y solo con stock, y ordenar por catálogo, precio, nombre o mayor descuento.
+3. Los criterios viajan en la URL (?q=&amp;categoria=&amp;min=&amp;max=&amp;oferta=1&amp;stock=1&amp;orden=): el enlace se puede compartir, la acción Atrás recupera el filtro anterior y un valor inválido se ignora.
+4. El texto y los precios se aplican al enviar el formulario; la categoría, el orden y las casillas, al cambiarlos. "Limpiar filtros" los borra.
+5. Un mínimo mayor que el máximo se avisa; sin coincidencias aparece un mensaje que sugiere cambiar la búsqueda o limpiar los filtros.</t>
+        </is>
+      </c>
+      <c r="H17" s="12" t="inlineStr">
+        <is>
+          <t>Solicitado</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="128" customHeight="1">
+      <c r="A18" s="12" t="inlineStr">
+        <is>
+          <t>RF-18</t>
+        </is>
+      </c>
+      <c r="B18" s="12" t="inlineStr">
+        <is>
+          <t>Ofertas y precio vigente</t>
+        </is>
+      </c>
+      <c r="C18" s="12" t="inlineStr">
+        <is>
+          <t>Funcional</t>
+        </is>
+      </c>
+      <c r="D18" s="12" t="inlineStr">
+        <is>
+          <t>Funcional de usuario</t>
+        </is>
+      </c>
+      <c r="E18" s="12" t="inlineStr">
+        <is>
+          <t>Cliente</t>
+        </is>
+      </c>
+      <c r="F18" s="12" t="inlineStr">
+        <is>
+          <t>El cliente debe poder ver qué productos están en oferta y cuánto cuestan con el descuento. Un producto con descuento mayor que 0 está en oferta; su precio vigente es el de lista menos el descuento, redondeado a pesos enteros, y es el que usan el carrito, el pago, las órdenes y los reportes.</t>
+        </is>
+      </c>
+      <c r="G18" s="12" t="inlineStr">
+        <is>
+          <t>1. Un producto con descuento mayor que 0 (entero, máximo 90) está en oferta; sin descuento, su precio vigente es el de lista.
+2. En oferta se muestran el precio vigente, el de lista tachado y el porcentaje de descuento; por ejemplo, con precio 10.000 y descuento 10 el precio vigente es 9.000. El carrito, el pago, las órdenes y los reportes usan siempre el precio vigente.
+3. La vista Ofertas lista solo los productos en oferta, de mayor a menor descuento, con los filtros de RF-17 salvo "solo ofertas".
+4. Sin productos en oferta aparece un aviso con el enlace al catálogo.</t>
+        </is>
+      </c>
+      <c r="H18" s="12" t="inlineStr">
+        <is>
+          <t>Solicitado</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="83" customHeight="1">
+      <c r="A19" s="12" t="inlineStr">
+        <is>
+          <t>RF-19</t>
+        </is>
+      </c>
+      <c r="B19" s="12" t="inlineStr">
+        <is>
+          <t>Ver productos por categoría</t>
+        </is>
+      </c>
+      <c r="C19" s="12" t="inlineStr">
+        <is>
+          <t>Funcional</t>
+        </is>
+      </c>
+      <c r="D19" s="12" t="inlineStr">
+        <is>
+          <t>Funcional de usuario</t>
+        </is>
+      </c>
+      <c r="E19" s="12" t="inlineStr">
+        <is>
+          <t>Cliente</t>
+        </is>
+      </c>
+      <c r="F19" s="12" t="inlineStr">
+        <is>
+          <t>El cliente debe poder recorrer el catálogo agrupado por categoría y abrir el listado de una categoría desde la barra lateral o desde la vista de categorías.</t>
+        </is>
+      </c>
+      <c r="G19" s="12" t="inlineStr">
+        <is>
+          <t>1. La vista Categorías agrupa los productos por categoría, con los tres primeros de cada una y el enlace "Ver los N productos".
+2. Una categoría sin productos muestra un aviso en lugar de un área en blanco.
+3. El listado de una categoría (?categoria=…) lleva su nombre por título; un código que no existe se ignora y se muestra todo el catálogo.</t>
+        </is>
+      </c>
+      <c r="H19" s="12" t="inlineStr">
+        <is>
+          <t>Solicitado</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="248" customHeight="1">
+      <c r="A20" s="12" t="inlineStr">
+        <is>
+          <t>RF-20</t>
+        </is>
+      </c>
+      <c r="B20" s="12" t="inlineStr">
+        <is>
+          <t>Pagar la compra</t>
+        </is>
+      </c>
+      <c r="C20" s="12" t="inlineStr">
+        <is>
+          <t>Funcional</t>
+        </is>
+      </c>
+      <c r="D20" s="12" t="inlineStr">
+        <is>
+          <t>Funcional de usuario</t>
+        </is>
+      </c>
+      <c r="E20" s="12" t="inlineStr">
+        <is>
+          <t>Cliente</t>
+        </is>
+      </c>
+      <c r="F20" s="12" t="inlineStr">
+        <is>
+          <t>El cliente debe poder pagar el contenido de su carrito indicando sus datos de envío y de pago, con o sin sesión iniciada. La entrega es a domicilio o con retiro en tienda; el costo de envío y el total se calculan al escoger la entrega.</t>
+        </is>
+      </c>
+      <c r="G20" s="12" t="inlineStr">
+        <is>
+          <t>1. Con el carrito vacío se avisa que no hay nada que pagar y no se muestra el formulario.
+2. Se puede comprar sin sesión; con sesión, los datos de envío se completan con los de la cuenta y se pueden cambiar para esa compra.
+3. Nombre, apellidos, correo (de dominio permitido, ver 1.3), región, comuna y dirección son requeridos y se validan al escribir.
+4. La entrega es a domicilio ($4.990, gratis desde $200.000 en productos) o con retiro en tienda (gratis); al escogerla se recalculan el envío, el total y el botón de pago.
+5. La tarjeta se valida (número de 13 a 19 dígitos con el algoritmo de Luhn, vencimiento no vencido y código de 3 o 4 dígitos); el número se agrupa de a cuatro al escribirlo y no se guarda.
+6. Un pedido de $0 (productos gratuitos con retiro en tienda) no pide tarjeta y su botón dice "Confirmar pedido".
+7. Antes de cobrar se revisa el stock; si falta, no se cobra y se nombran los productos sin unidades suficientes.</t>
+        </is>
+      </c>
+      <c r="H20" s="12" t="inlineStr">
+        <is>
+          <t>Solicitado</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="158" customHeight="1">
+      <c r="A21" s="12" t="inlineStr">
+        <is>
+          <t>RF-21</t>
+        </is>
+      </c>
+      <c r="B21" s="12" t="inlineStr">
+        <is>
+          <t>Confirmar o rechazar el pago</t>
+        </is>
+      </c>
+      <c r="C21" s="12" t="inlineStr">
+        <is>
+          <t>Funcional</t>
+        </is>
+      </c>
+      <c r="D21" s="12" t="inlineStr">
+        <is>
+          <t>Funcional de sistema</t>
+        </is>
+      </c>
+      <c r="E21" s="12" t="inlineStr">
+        <is>
+          <t>Cliente</t>
+        </is>
+      </c>
+      <c r="F21" s="12" t="inlineStr">
+        <is>
+          <t>El sistema debe aprobar o rechazar el pago simulado según el número de la tarjeta y mostrar al cliente el resultado, sin cobro ni cambios en el stock ni en el carrito cuando el pago se rechaza.</t>
+        </is>
+      </c>
+      <c r="G21" s="12" t="inlineStr">
+        <is>
+          <t>1. El número 4242 4242 4242 4242 se aprueba, el 4000 0000 0000 0002 lo rechaza el emisor y el 4000 0000 0000 9995 se rechaza por fondos insuficientes; cualquier otro número válido se aprueba.
+2. Si se aprueba, se crea la orden (RF-22), se vacía el carrito y se muestra la confirmación de /pago/correcto/:numero con la boleta como resumen.
+3. Si se rechaza, /pago/error muestra el motivo y el resumen del pedido: no hay cobro, el stock y el carrito no cambian, y "Reintentar el pago" vuelve al pago con los datos de envío (la tarjeta no se conserva).
+4. La confirmación solo la ve quien puede ver esa orden; en cualquier otro caso aparece "Orden no encontrada", sin revelar si existe.</t>
+        </is>
+      </c>
+      <c r="H21" s="12" t="inlineStr">
+        <is>
+          <t>Solicitado</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="143" customHeight="1">
+      <c r="A22" s="12" t="inlineStr">
+        <is>
+          <t>RF-22</t>
+        </is>
+      </c>
+      <c r="B22" s="12" t="inlineStr">
+        <is>
+          <t>Registrar la orden y mostrar la boleta</t>
+        </is>
+      </c>
+      <c r="C22" s="12" t="inlineStr">
+        <is>
+          <t>Funcional</t>
+        </is>
+      </c>
+      <c r="D22" s="12" t="inlineStr">
+        <is>
+          <t>Funcional de sistema</t>
+        </is>
+      </c>
+      <c r="E22" s="12" t="inlineStr">
+        <is>
+          <t>Cliente, Administrador, Administrador logístico</t>
+        </is>
+      </c>
+      <c r="F22" s="12" t="inlineStr">
+        <is>
+          <t>Cada pago aprobado debe registrar una orden con su detalle, descontar el stock de los productos comprados y poder mostrarse como boleta. La orden conserva los precios vigentes al momento de la compra.</t>
+        </is>
+      </c>
+      <c r="G22" s="12" t="inlineStr">
+        <is>
+          <t>1. Cada compra aprobada crea una orden ORD-AAAA-NNNN, correlativa dentro del año, con los datos del comprador, la entrega, el costo de envío, el medio de pago ("Tarjeta terminada en NNNN") y un ítem por producto con su precio vigente.
+2. La orden descuenta el stock de cada producto y se valida entera antes de escribir: si algo falla, no cambia nada.
+3. La boleta muestra el comprador (RUN o invitado), la entrega, el medio de pago, el detalle, el subtotal, el envío y el total con el IVA desglosado (neto más 19 %); es un comprobante simulado y se puede imprimir.
+4. Una orden conserva su detalle aunque el producto se elimine del catálogo.</t>
+        </is>
+      </c>
+      <c r="H22" s="12" t="inlineStr">
+        <is>
+          <t>Solicitado</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="143" customHeight="1">
+      <c r="A23" s="12" t="inlineStr">
+        <is>
+          <t>RF-23</t>
+        </is>
+      </c>
+      <c r="B23" s="12" t="inlineStr">
+        <is>
+          <t>Gestionar mi perfil</t>
+        </is>
+      </c>
+      <c r="C23" s="12" t="inlineStr">
+        <is>
+          <t>Funcional</t>
+        </is>
+      </c>
+      <c r="D23" s="12" t="inlineStr">
+        <is>
+          <t>Funcional de usuario</t>
+        </is>
+      </c>
+      <c r="E23" s="12" t="inlineStr">
+        <is>
+          <t>Cliente, Administrador, Administrador logístico</t>
+        </is>
+      </c>
+      <c r="F23" s="12" t="inlineStr">
+        <is>
+          <t>El usuario con sesión iniciada debe poder ver y editar sus datos y cambiar su contraseña.</t>
+        </is>
+      </c>
+      <c r="G23" s="12" t="inlineStr">
+        <is>
+          <t>1. El perfil muestra el RUN y el tipo de usuario, que no se pueden editar.
+2. Permite editar nombre, apellidos, correo, fecha de nacimiento, región, comuna y dirección con las validaciones de RF-01; un correo usado por otra cuenta se rechaza.
+3. Al guardar, el saludo del encabezado se actualiza sin cerrar sesión.
+4. El cambio de contraseña pide la actual, la nueva y su repetición; se rechaza si la actual es incorrecta, si la nueva y su repetición no coinciden o si la nueva es igual a la actual.
+5. El Administrador y el Administrador logístico ven el perfil dentro del panel (/admin/perfil).</t>
+        </is>
+      </c>
+      <c r="H23" s="12" t="inlineStr">
+        <is>
+          <t>Solicitado</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="98" customHeight="1">
+      <c r="A24" s="12" t="inlineStr">
+        <is>
+          <t>RF-24</t>
+        </is>
+      </c>
+      <c r="B24" s="12" t="inlineStr">
+        <is>
+          <t>Consultar el historial de compras</t>
+        </is>
+      </c>
+      <c r="C24" s="12" t="inlineStr">
+        <is>
+          <t>Funcional</t>
+        </is>
+      </c>
+      <c r="D24" s="12" t="inlineStr">
+        <is>
+          <t>Funcional de usuario</t>
+        </is>
+      </c>
+      <c r="E24" s="12" t="inlineStr">
+        <is>
+          <t>Cliente</t>
+        </is>
+      </c>
+      <c r="F24" s="12" t="inlineStr">
+        <is>
+          <t>El cliente con sesión iniciada debe poder consultar sus compras anteriores y abrir la boleta de cada una.</t>
+        </is>
+      </c>
+      <c r="G24" s="12" t="inlineStr">
+        <is>
+          <t>1. /mis-compras exige sesión y lista las compras de la cuenta, de la más reciente a la más antigua, con número, fecha, productos y total, más la cantidad de compras y el gasto total.
+2. Sin compras, avisa y enlaza al catálogo.
+3. /mis-compras/:numero muestra la boleta de una compra propia; la de otra cuenta o la de un invitado aparece como "Orden no encontrada".</t>
+        </is>
+      </c>
+      <c r="H24" s="12" t="inlineStr">
+        <is>
+          <t>Solicitado</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="143" customHeight="1">
+      <c r="A25" s="12" t="inlineStr">
+        <is>
+          <t>RF-25</t>
+        </is>
+      </c>
+      <c r="B25" s="12" t="inlineStr">
+        <is>
+          <t>Mantenedor de Categorías</t>
+        </is>
+      </c>
+      <c r="C25" s="12" t="inlineStr">
+        <is>
+          <t>Funcional</t>
+        </is>
+      </c>
+      <c r="D25" s="12" t="inlineStr">
+        <is>
+          <t>Funcional de usuario</t>
+        </is>
+      </c>
+      <c r="E25" s="12" t="inlineStr">
+        <is>
+          <t>Administrador</t>
+        </is>
+      </c>
+      <c r="F25" s="12" t="inlineStr">
+        <is>
+          <t>El administrador debe poder listar, crear, editar y eliminar las categorías del catálogo, con código (requerido, de 3 a 30 caracteres entre minúsculas, números y guiones, único) y nombre (requerido, máx. 50). Las categorías que forman parte del asistente de armado (RF-07) no pueden eliminarse.</t>
+        </is>
+      </c>
+      <c r="G25" s="12" t="inlineStr">
+        <is>
+          <t>1. El listado muestra el código, el nombre, el paso del asistente y el número de productos de cada categoría, con las acciones de crear, editar y eliminar.
+2. Se rechazan un código fuera de 3 a 30 caracteres, con caracteres no permitidos o repetido, y un nombre vacío o de más de 50 caracteres; el código no cambia al editar.
+3. Las categorías nuevas aparecen en el catálogo, en los filtros y en la ficha de producto; no participan del asistente de armado.
+4. Eliminar pide confirmación y se rechaza si la categoría es un paso del asistente o tiene productos.</t>
+        </is>
+      </c>
+      <c r="H25" s="12" t="inlineStr">
+        <is>
+          <t>Solicitado</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="98" customHeight="1">
+      <c r="A26" s="12" t="inlineStr">
+        <is>
+          <t>RF-26</t>
+        </is>
+      </c>
+      <c r="B26" s="12" t="inlineStr">
+        <is>
+          <t>Productos críticos</t>
+        </is>
+      </c>
+      <c r="C26" s="12" t="inlineStr">
+        <is>
+          <t>Funcional</t>
+        </is>
+      </c>
+      <c r="D26" s="12" t="inlineStr">
+        <is>
+          <t>Funcional de sistema</t>
+        </is>
+      </c>
+      <c r="E26" s="12" t="inlineStr">
+        <is>
+          <t>Administrador, Administrador logístico</t>
+        </is>
+      </c>
+      <c r="F26" s="12" t="inlineStr">
+        <is>
+          <t>El administrador y el administrador logístico deben poder ver qué productos tienen un stock igual o inferior a su stock crítico, para decidir su reposición.</t>
+        </is>
+      </c>
+      <c r="G26" s="12" t="inlineStr">
+        <is>
+          <t>1. La vista lista los productos con stock igual o inferior a su stock crítico: primero los agotados, luego los de mayor faltante y, a igualdad, por código.
+2. Cada fila muestra el stock, el umbral, las unidades que faltan y el estado.
+3. El Administrador accede desde cada fila a la ficha del producto para reponer; el Administrador logístico la ve en modo lectura.
+4. Sin productos críticos, la vista lo indica.</t>
+        </is>
+      </c>
+      <c r="H26" s="12" t="inlineStr">
+        <is>
+          <t>Solicitado</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="128" customHeight="1">
+      <c r="A27" s="12" t="inlineStr">
+        <is>
+          <t>RF-27</t>
+        </is>
+      </c>
+      <c r="B27" s="12" t="inlineStr">
+        <is>
+          <t>Reportes</t>
+        </is>
+      </c>
+      <c r="C27" s="12" t="inlineStr">
+        <is>
+          <t>Funcional</t>
+        </is>
+      </c>
+      <c r="D27" s="12" t="inlineStr">
+        <is>
+          <t>Funcional de usuario</t>
+        </is>
+      </c>
+      <c r="E27" s="12" t="inlineStr">
+        <is>
+          <t>Administrador</t>
+        </is>
+      </c>
+      <c r="F27" s="12" t="inlineStr">
+        <is>
+          <t>El administrador debe poder consultar reportes de las ventas del periodo que escoja y del inventario.</t>
+        </is>
+      </c>
+      <c r="G27" s="12" t="inlineStr">
+        <is>
+          <t>1. Permite acotar el periodo con fechas desde y hasta, ambas inclusivas; un rango invertido se avisa.
+2. Resume las órdenes, los ingresos (ítems más envío, con IVA), los envíos, las unidades y el ticket promedio del periodo.
+3. Muestra las ventas por mes y por categoría, los 5 productos más vendidos y los 5 clientes que más gastaron (un invitado se agrupa por su correo).
+4. Muestra el inventario valorizado a precio de lista y cuántos productos están en stock crítico.</t>
+        </is>
+      </c>
+      <c r="H27" s="12" t="inlineStr">
+        <is>
+          <t>Solicitado</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="143" customHeight="1">
+      <c r="A28" s="12" t="inlineStr">
+        <is>
           <t>RNF-01</t>
         </is>
       </c>
-      <c r="B17" s="12" t="inlineStr">
+      <c r="B28" s="12" t="inlineStr">
         <is>
           <t>Rendimiento: carga de cada vista en menos de 2 segundos</t>
         </is>
       </c>
-      <c r="C17" s="12" t="inlineStr">
+      <c r="C28" s="12" t="inlineStr">
         <is>
           <t>No Funcional</t>
         </is>
       </c>
-      <c r="D17" s="12" t="inlineStr">
+      <c r="D28" s="12" t="inlineStr">
         <is>
           <t>No funcional de producto</t>
         </is>
       </c>
-      <c r="E17" s="12" t="inlineStr">
+      <c r="E28" s="12" t="inlineStr">
         <is>
           <t>Cliente, Administrador logístico, Administrador</t>
         </is>
       </c>
-      <c r="F17" s="12" t="inlineStr">
-        <is>
-          <t>Al tratarse de un sitio estático sin backend, cada vista debe cargar completamente en menos de 2 segundos en una conexión de banda ancha estándar, dado que no existen llamadas a servicios externos ni consultas a base de datos en esta entrega.</t>
-        </is>
-      </c>
-      <c r="G17" s="12" t="inlineStr">
-        <is>
-          <t>1. Servido por HTTP en una conexión de banda ancha estándar, cualquier vista termina de cargar en menos de 2 segundos, medido en la pestaña de red del navegador con la caché deshabilitada.
-2. Al cargar cualquier vista, las únicas peticiones registradas son de recursos del mismo origen (HTML de secciones, CSS, JS e imágenes); no se observan llamadas a servicios externos.
-3. La composición de secciones mediante fetch() se completa antes de que el usuario pueda interactuar, sin dejar contenedores vacíos de forma permanente.</t>
-        </is>
-      </c>
-      <c r="H17" s="12" t="inlineStr">
-        <is>
-          <t>Solicitado</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="259" customHeight="1">
-      <c r="A18" s="12" t="inlineStr">
+      <c r="F28" s="12" t="inlineStr">
+        <is>
+          <t>Al ser una aplicación sin backend, que no consulta servicios externos ni bases de datos, cada vista debe cargar completamente en menos de 2 segundos en una conexión de banda ancha estándar, y el cambio entre vistas no debe recargar la página.</t>
+        </is>
+      </c>
+      <c r="G28" s="12" t="inlineStr">
+        <is>
+          <t>1. Servida con npm run dev o npm run preview en una conexión de banda ancha estándar y con la caché deshabilitada, cualquier vista termina de cargar en menos de 2 segundos, medido en la pestaña de red del navegador. El empaquetado de producción pesa 432 kB de JavaScript (125 kB comprimido) y 242 kB de CSS (34 kB comprimido).
+2. Al cargar cualquier vista, las únicas peticiones registradas son de recursos del mismo origen (JavaScript, CSS e imágenes); no se observan llamadas a servicios externos.
+3. El cambio entre vistas lo resuelve el enrutador del cliente, sin recargar la página.</t>
+        </is>
+      </c>
+      <c r="H28" s="12" t="inlineStr">
+        <is>
+          <t>Solicitado</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="278" customHeight="1">
+      <c r="A29" s="12" t="inlineStr">
         <is>
           <t>RNF-02</t>
         </is>
       </c>
-      <c r="B18" s="12" t="inlineStr">
+      <c r="B29" s="12" t="inlineStr">
         <is>
           <t>Seguridad: control de acceso por rol, enmascarado de contraseñas y validación de formularios</t>
         </is>
       </c>
-      <c r="C18" s="12" t="inlineStr">
+      <c r="C29" s="12" t="inlineStr">
         <is>
           <t>No Funcional</t>
         </is>
       </c>
-      <c r="D18" s="12" t="inlineStr">
+      <c r="D29" s="12" t="inlineStr">
         <is>
           <t>No funcional de producto</t>
         </is>
       </c>
-      <c r="E18" s="12" t="inlineStr">
+      <c r="E29" s="12" t="inlineStr">
         <is>
           <t>Cliente, Administrador logístico, Administrador</t>
         </is>
       </c>
-      <c r="F18" s="12" t="inlineStr">
-        <is>
-          <t>• Todas las contraseñas ingresadas en los formularios deben enmascararse (tipo password) en pantalla, tanto en el inicio de sesión como en el registro y en el mantenedor de Usuarios.
+      <c r="F29" s="12" t="inlineStr">
+        <is>
+          <t>• Todas las contraseñas ingresadas en los formularios deben enmascararse (tipo password) en pantalla, tanto en el inicio de sesión como en el registro, el perfil y el mantenedor de Usuarios; lo mismo vale para el código de seguridad de la tarjeta en el pago.
 • Las vistas del panel administrativo deben quedar inaccesibles para un usuario sin sesión iniciada y para un usuario autenticado con rol Cliente, cuyo acceso se limita a la tienda pública.
-• Las funcionalidades visibles para el rol Administrador logístico deben restringirse a productos y órdenes en modo lectura; el resto de opciones administrativas no debe renderizarse para este rol.
+• Las funcionalidades visibles para el rol Administrador logístico deben restringirse a productos, productos críticos y órdenes en modo lectura, y a su propio perfil; el resto de opciones administrativas no debe renderizarse para este rol.
 • El cierre de sesión (RF-13) debe limpiar los datos de sesión del cliente, de modo que las vistas administrativas dejen de ser accesibles.
-• Todos los formularios (registro, login, contacto, producto, usuario) deben validarse en tiempo real en el cliente, mostrando mensajes de error personalizados antes de permitir el envío.
+• Todos los formularios (registro, login, contacto, pago, perfil, producto, categoría, usuario) deben validarse en tiempo real en el cliente, mostrando mensajes de error personalizados antes de permitir el envío.
 • Además del mensaje de error, cada campo validado debe ofrecer una sugerencia que anticipe el formato esperado —por ejemplo el del RUN o los dominios de correo aceptados—, visible antes de que el usuario cometa el error.</t>
         </is>
       </c>
-      <c r="G18" s="12" t="inlineStr">
+      <c r="G29" s="12" t="inlineStr">
         <is>
           <t>1. Intentar abrir una vista administrativa por URL directa redirige al inicio de sesión sin sesión iniciada, y deniega el acceso con rol Cliente o tras haber cerrado sesión (RF-13).
-2. Dado un usuario autenticado con rol Administrador logístico, el menú administrativo solo contiene Productos y Órdenes: las demás opciones no están presentes en el DOM, no basta con ocultarlas por CSS.
-3. Todo campo de contraseña del sistema (inicio de sesión, registro y mantenedor de Usuarios) tiene el atributo type="password", verificable inspeccionando el DOM.
+2. Dado un usuario autenticado con rol Administrador logístico, el menú administrativo solo contiene Productos, Críticos, Órdenes y Mi perfil: las demás opciones no están presentes en el DOM, no basta con ocultarlas por CSS.
+3. Todo campo de contraseña del sistema y el código de seguridad de la tarjeta tienen el atributo type="password", verificable inspeccionando el DOM.
 4. En cualquier formulario, un valor inválido muestra su mensaje de error antes de pulsar el botón de envío.
 5. Cada campo con reglas de formato (RUN, correo, contraseña) muestra una sugerencia con el formato esperado antes de cualquier intento de envío, distinta del mensaje de error que aparece al infringirlo.
-6. Dado un usuario autenticado con rol Administrador logístico, abrir por URL directa un mantenedor de creación o edición deniega el acceso y no renderiza la vista.</t>
-        </is>
-      </c>
-      <c r="H18" s="12" t="inlineStr">
-        <is>
-          <t>Solicitado</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="124" customHeight="1">
-      <c r="A19" s="12" t="inlineStr">
+6. Dado un usuario autenticado con rol Administrador logístico, abrir por URL directa un formulario de creación o edición deniega el acceso y no renderiza la vista.
+7. Tras iniciar sesión, solo se respeta como destino una ruta del mismo sitio.</t>
+        </is>
+      </c>
+      <c r="H29" s="12" t="inlineStr">
+        <is>
+          <t>Solicitado</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="143" customHeight="1">
+      <c r="A30" s="12" t="inlineStr">
         <is>
           <t>RNF-03</t>
         </is>
       </c>
-      <c r="B19" s="12" t="inlineStr">
-        <is>
-          <t>Fiabilidad: navegación sin errores de carga ni de JavaScript</t>
-        </is>
-      </c>
-      <c r="C19" s="12" t="inlineStr">
+      <c r="B30" s="12" t="inlineStr">
+        <is>
+          <t>Fiabilidad: navegación sin errores y recuperación de un almacenamiento corrupto</t>
+        </is>
+      </c>
+      <c r="C30" s="12" t="inlineStr">
         <is>
           <t>No Funcional</t>
         </is>
       </c>
-      <c r="D19" s="12" t="inlineStr">
+      <c r="D30" s="12" t="inlineStr">
         <is>
           <t>No funcional de producto</t>
         </is>
       </c>
-      <c r="E19" s="12" t="inlineStr">
+      <c r="E30" s="12" t="inlineStr">
         <is>
           <t>Cliente, Administrador logístico, Administrador</t>
         </is>
       </c>
-      <c r="F19" s="12" t="inlineStr">
-        <is>
-          <t>Al no depender de un backend, el sistema no debe presentar errores de carga de página bajo uso normal del navegador; los únicos incidentes esperables son errores de validación de formularios, que deben gestionarse y comunicarse claramente al usuario sin interrumpir la navegación.</t>
-        </is>
-      </c>
-      <c r="G19" s="12" t="inlineStr">
+      <c r="F30" s="12" t="inlineStr">
+        <is>
+          <t>Al no depender de un backend, el sistema no debe presentar errores de carga de página bajo uso normal del navegador; los únicos incidentes esperables son errores de validación de formularios, que deben gestionarse y comunicarse claramente al usuario sin interrumpir la navegación, y un almacenamiento del navegador corrupto, bloqueado o lleno, del que la aplicación debe recuperarse.</t>
+        </is>
+      </c>
+      <c r="G30" s="12" t="inlineStr">
         <is>
           <t>1. Navegando por todas las vistas del sitio, la consola del navegador no registra errores de JavaScript.
-2. Un archivo de sección que no se puede cargar deja el error en la consola y el resto de la página utilizable, según el manejo de errores implementado en src/scripts/includes.js.
-3. Un error de validación se comunica junto al campo afectado y la navegación del sitio sigue disponible.
-4. Un contenido inválido o corrupto en localStorage hace que el carrito se inicialice vacío, en lugar de interrumpir la ejecución.</t>
-        </is>
-      </c>
-      <c r="H19" s="12" t="inlineStr">
-        <is>
-          <t>Solicitado</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="79" customHeight="1">
-      <c r="A20" s="12" t="inlineStr">
+2. Un error de validación se comunica junto al campo afectado y la navegación del sitio sigue disponible.
+3. Un contenido inválido o corrupto en localStorage hace que el carrito se inicialice vacío, en lugar de interrumpir la ejecución; una sesión corrupta se trata como sin sesión y una colección corrupta vuelve a su semilla.
+4. Si el almacenamiento está bloqueado o lleno, el error queda en la consola y la aplicación sigue siendo utilizable.</t>
+        </is>
+      </c>
+      <c r="H30" s="12" t="inlineStr">
+        <is>
+          <t>Solicitado</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="83" customHeight="1">
+      <c r="A31" s="12" t="inlineStr">
         <is>
           <t>RNF-04</t>
         </is>
       </c>
-      <c r="B20" s="12" t="inlineStr">
+      <c r="B31" s="12" t="inlineStr">
         <is>
           <t>Disponibilidad: sitio accesible mediante el hosting elegido</t>
         </is>
       </c>
-      <c r="C20" s="12" t="inlineStr">
+      <c r="C31" s="12" t="inlineStr">
         <is>
           <t>No Funcional</t>
         </is>
       </c>
-      <c r="D20" s="12" t="inlineStr">
+      <c r="D31" s="12" t="inlineStr">
         <is>
           <t>No funcional Externos</t>
         </is>
       </c>
-      <c r="E20" s="12" t="inlineStr">
+      <c r="E31" s="12" t="inlineStr">
         <is>
           <t>Cliente, Administrador logístico, Administrador</t>
         </is>
       </c>
-      <c r="F20" s="12" t="inlineStr">
-        <is>
-          <t>Al ser un sitio 100% estático, sin servidor de aplicación ni base de datos, la disponibilidad depende únicamente del servicio de hosting o repositorio utilizado para publicarlo. El proyecto no compromete un porcentaje propio de disponibilidad: el exigible es el que ofrezca el hosting elegido, ya que ningún componente del sistema puede degradarla.</t>
-        </is>
-      </c>
-      <c r="G20" s="12" t="inlineStr">
+      <c r="F31" s="12" t="inlineStr">
+        <is>
+          <t>Al publicarse como archivos estáticos (la carpeta dist/ que genera npm run build), sin servidor de aplicación ni base de datos, la disponibilidad depende únicamente del servicio de hosting o repositorio utilizado para publicarlo. El proyecto no compromete un porcentaje propio de disponibilidad: el exigible es el que ofrezca el hosting elegido, ya que ningún componente del sistema puede degradarla.</t>
+        </is>
+      </c>
+      <c r="G31" s="12" t="inlineStr">
         <is>
           <t>1. Publicado en el servicio de hosting o repositorio elegido, el sitio es accesible mediante su URL pública sin requerir credenciales.</t>
         </is>
       </c>
-      <c r="H20" s="12" t="inlineStr">
-        <is>
-          <t>Solicitado</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="259" customHeight="1">
-      <c r="A21" s="12" t="inlineStr">
+      <c r="H31" s="12" t="inlineStr">
+        <is>
+          <t>Solicitado</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="248" customHeight="1">
+      <c r="A32" s="12" t="inlineStr">
         <is>
           <t>RNF-05</t>
         </is>
       </c>
-      <c r="B21" s="12" t="inlineStr">
-        <is>
-          <t>Mantenibilidad: secciones HTML separadas, CSS externo único y HTML5 semántico válido</t>
-        </is>
-      </c>
-      <c r="C21" s="12" t="inlineStr">
+      <c r="B32" s="12" t="inlineStr">
+        <is>
+          <t>Mantenibilidad: componentes React de responsabilidad única, CSS externo único, HTML5 semántico y ESLint</t>
+        </is>
+      </c>
+      <c r="C32" s="12" t="inlineStr">
         <is>
           <t>No Funcional</t>
         </is>
       </c>
-      <c r="D21" s="12" t="inlineStr">
+      <c r="D32" s="12" t="inlineStr">
         <is>
           <t>No funcional de producto</t>
         </is>
       </c>
-      <c r="E21" s="12" t="inlineStr">
+      <c r="E32" s="12" t="inlineStr">
         <is>
           <t>Desarrollador</t>
         </is>
       </c>
-      <c r="F21" s="12" t="inlineStr">
-        <is>
-          <t>El sitio debe mantenerse mediante la separación de cada sección de la página (encabezado, navegación, aside, cuerpo, pie de página) en archivos HTML independientes referenciados desde index.html, y mediante una hoja de estilos CSS externa única. El mantenimiento —agregar productos de prueba, ajustar validaciones— lo realiza directamente el desarrollador editando estos archivos, bajo demanda y sin ventanas programadas, dado que el sitio no almacena datos de producción que obliguen a detenerlo.
-Cada vista debe construirse con etiquetado HTML5 semántico —&lt;header&gt;, &lt;nav&gt;, &lt;main&gt;, &lt;section&gt;, &lt;article&gt; y &lt;footer&gt;— en lugar de contenedores &lt;div&gt; genéricos, de modo que la estructura del documento sea autodescriptiva y las secciones compartidas puedan reemplazarse sin ambigüedad. El contenido textual debe estructurarse con una jerarquía de encabezados, párrafos y listas, y no con saltos de línea o estilos que los imiten. Cada control de formulario debe tener su etiqueta &lt;label&gt; asociada mediante el atributo for y declarar el atributo autocomplete que corresponda al dato solicitado. El comportamiento de las validaciones se especifica en 3.3.2, y el marcado de cada vista debe validar sin errores contra el validador del W3C.</t>
-        </is>
-      </c>
-      <c r="G21" s="12" t="inlineStr">
-        <is>
-          <t>1. Cada sección de la página (encabezado, navegación, aside, cuerpo y pie) reside en su propio archivo dentro de src/pages/ y se referencia desde index.html mediante el atributo data-include.
-2. Existe una única hoja de estilos propia y externa (src/styles/style.css), y ninguna vista define estilos mediante atributos style ni bloques &lt;style&gt;.
-3. Al modificar una sección compartida (por ejemplo el pie de página), el cambio se refleja en todas las vistas habiendo editado un solo archivo.
+      <c r="F32" s="12" t="inlineStr">
+        <is>
+          <t>El código debe organizarse en componentes React de responsabilidad única que reciben sus datos por props (components/ y pages/), hooks reutilizables (hooks/), reglas de negocio puras, sin DOM ni almacenamiento (logic/ y utils/), y una hoja de estilos CSS externa única. Los componentes compartidos —encabezado, menú, barra lateral y pie de página— residen en un solo archivo cada uno. El mantenimiento —agregar productos de prueba, ajustar validaciones— lo realiza directamente el desarrollador editando estos archivos, bajo demanda y sin ventanas programadas, dado que el sitio no almacena datos de producción que obliguen a detenerlo.
+Cada vista debe construirse con etiquetado HTML5 semántico —&lt;header&gt;, &lt;nav&gt;, &lt;main&gt;, &lt;section&gt;, &lt;article&gt; y &lt;footer&gt;— en lugar de contenedores &lt;div&gt; genéricos, de modo que la estructura del documento sea autodescriptiva. El contenido textual debe estructurarse con una jerarquía de encabezados, párrafos y listas, y no con saltos de línea o estilos que los imiten. Cada control de formulario debe tener su etiqueta &lt;label&gt; asociada mediante el atributo for y declarar el atributo autocomplete que corresponda al dato solicitado. El comportamiento de las validaciones se especifica en 3.3.2, y el código debe pasar el análisis de ESLint sin errores.</t>
+        </is>
+      </c>
+      <c r="G32" s="12" t="inlineStr">
+        <is>
+          <t>1. Cada componente tiene una sola responsabilidad y recibe sus datos por props; las reglas de negocio viven en src/logic/ y src/utils/, sin DOM ni almacenamiento.
+2. Existe una única hoja de estilos propia y externa (src/styles/style.css), y ninguna vista define estilos mediante atributos style.
+3. Al modificar un componente compartido (por ejemplo, el pie de página), el cambio se refleja en todas las vistas habiendo editado un solo archivo.
 4. Inspeccionando el marcado de cualquier vista, la estructura se expresa con &lt;header&gt;, &lt;nav&gt;, &lt;main&gt;, &lt;section&gt;/&lt;article&gt; y &lt;footer&gt;, y no con contenedores &lt;div&gt; genéricos en su lugar; cada vista tiene un único &lt;h1&gt; y su contenido textual se estructura con encabezados, párrafos y listas.
 5. Cada control de formulario tiene una etiqueta &lt;label&gt; asociada mediante un atributo for que coincide con el id del campo.
 6. Los campos de formulario declaran el atributo autocomplete con el valor que corresponde al dato solicitado.
-7. El marcado de cada vista, servido por HTTP, pasa el validador del W3C (validator.w3.org) sin errores.</t>
-        </is>
-      </c>
-      <c r="H21" s="12" t="inlineStr">
-        <is>
-          <t>Solicitado</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="109" customHeight="1">
-      <c r="A22" s="12" t="inlineStr">
+7. npm run lint termina sin errores.</t>
+        </is>
+      </c>
+      <c r="H32" s="12" t="inlineStr">
+        <is>
+          <t>Solicitado</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="98" customHeight="1">
+      <c r="A33" s="12" t="inlineStr">
         <is>
           <t>RNF-06</t>
         </is>
       </c>
-      <c r="B22" s="12" t="inlineStr">
-        <is>
-          <t>Portabilidad: funcionamiento en navegadores modernos servido por HTTP</t>
-        </is>
-      </c>
-      <c r="C22" s="12" t="inlineStr">
+      <c r="B33" s="12" t="inlineStr">
+        <is>
+          <t>Portabilidad: navegadores modernos y Node.js 22.22 o superior</t>
+        </is>
+      </c>
+      <c r="C33" s="12" t="inlineStr">
         <is>
           <t>No Funcional</t>
         </is>
       </c>
-      <c r="D22" s="12" t="inlineStr">
+      <c r="D33" s="12" t="inlineStr">
         <is>
           <t>No funcional de producto</t>
         </is>
       </c>
-      <c r="E22" s="12" t="inlineStr">
+      <c r="E33" s="12" t="inlineStr">
         <is>
           <t>Cliente, Administrador logístico, Administrador</t>
         </is>
       </c>
-      <c r="F22" s="12" t="inlineStr">
-        <is>
-          <t>El sistema debe funcionar correctamente en cualquier navegador web moderno (Chrome, Firefox, Edge) sin depender de un sistema operativo, compilador o plataforma de desarrollo específica, dado que utiliza únicamente HTML, CSS, JavaScript y Bootstrap. La única condición de ejecución es servirlo mediante un servidor HTTP (ver 3.1.4).</t>
-        </is>
-      </c>
-      <c r="G22" s="12" t="inlineStr">
-        <is>
-          <t>1. Servido por HTTP, el sitio se visualiza y opera correctamente en las versiones actuales de Chrome, Firefox y Edge; abierto con el esquema file:// las secciones no se cargan (ver 3.1.4).
-2. El proyecto no requiere compilación, instalación de dependencias ni configuración específica del sistema operativo para ejecutarse.
+      <c r="F33" s="12" t="inlineStr">
+        <is>
+          <t>El sistema debe funcionar correctamente en cualquier navegador web moderno (Chrome, Firefox, Edge) sin depender de un sistema operativo o plataforma de desarrollo específica, dado que utiliza únicamente HTML, CSS, JavaScript, React y Bootstrap. Para ejecutarlo localmente o generar su versión de producción se requiere Node.js 22.22 o superior (ver 3.1.4).</t>
+        </is>
+      </c>
+      <c r="G33" s="12" t="inlineStr">
+        <is>
+          <t>1. El sitio se visualiza y opera correctamente en las versiones actuales de Chrome, Firefox y Edge, servido con npm run dev o desde la carpeta dist/.
+2. El proyecto requiere Node.js 22.22 o superior; se instala con npm install y se empaqueta con npm run build, sin configuración específica del sistema operativo.
 3. En cualquier viewport de escritorio, tablet o móvil el diseño se adapta sin producir desplazamiento horizontal (ver 3.1.2).</t>
         </is>
       </c>
-      <c r="H22" s="12" t="inlineStr">
-        <is>
-          <t>Solicitado</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="199" customHeight="1">
-      <c r="A23" s="12" t="inlineStr">
+      <c r="H33" s="12" t="inlineStr">
+        <is>
+          <t>Solicitado</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="188" customHeight="1">
+      <c r="A34" s="12" t="inlineStr">
         <is>
           <t>RNF-07</t>
         </is>
       </c>
-      <c r="B23" s="12" t="inlineStr">
-        <is>
-          <t>Otros requisitos: repositorio GitHub público y entregables de la Entrega I</t>
-        </is>
-      </c>
-      <c r="C23" s="12" t="inlineStr">
+      <c r="B34" s="12" t="inlineStr">
+        <is>
+          <t>Otros requisitos: repositorio GitHub público y entregables de la Entrega II</t>
+        </is>
+      </c>
+      <c r="C34" s="12" t="inlineStr">
         <is>
           <t>No Funcional</t>
         </is>
       </c>
-      <c r="D23" s="12" t="inlineStr">
+      <c r="D34" s="12" t="inlineStr">
         <is>
           <t>No funcional de la Organización</t>
         </is>
       </c>
-      <c r="E23" s="12" t="inlineStr">
+      <c r="E34" s="12" t="inlineStr">
         <is>
           <t>Desarrollador, Docente evaluador</t>
         </is>
       </c>
-      <c r="F23" s="12" t="inlineStr">
-        <is>
-          <t>• El proyecto debe mantenerse en un repositorio Git/GitHub público, con historial de commits claros y coherentes que documenten el avance del desarrollo, ya que este historial será evaluado como parte de la ronda de preguntas de la Entrega I.
+      <c r="F34" s="12" t="inlineStr">
+        <is>
+          <t>• El proyecto debe mantenerse en un repositorio Git/GitHub público, con historial de commits claros y coherentes que documenten el avance del desarrollo, ya que este historial será evaluado como parte de la ronda de preguntas de la Entrega II.
 • El repositorio debe documentar cómo ejecutar el proyecto localmente (ver 3.1.4), que es un prerrequisito de ejecución y no una comodidad.
 • El proyecto es desarrollado de forma individual por un único estudiante, modalidad autorizada por el docente de la asignatura; en consecuencia, el historial del repositorio refleja el avance de un solo autor y no una distribución de tareas entre integrantes de un equipo.
-• Además del enlace al repositorio público, la entrega incluye el proyecto frontend comprimido y este documento ERS, conforme a los entregables definidos en el Anexo 1 y en la pauta de la Evaluación Parcial N° 1.</t>
-        </is>
-      </c>
-      <c r="G23" s="12" t="inlineStr">
+• Además del enlace al repositorio público, la entrega incluye el proyecto frontend comprimido y este documento ERS en su última versión, conforme a los entregables definidos en el Anexo 1 y en la pauta de la Evaluación Parcial N° 2.</t>
+        </is>
+      </c>
+      <c r="G34" s="12" t="inlineStr">
         <is>
           <t>1. El repositorio Git/GitHub del proyecto es público y accesible mediante su URL sin requerir credenciales.
-2. Los commits documentan el avance del desarrollo con mensajes claros y coherentes, verificables en la ronda de preguntas de la Entrega I.
-3. El repositorio documenta cómo ejecutar el proyecto localmente (python3 -m http.server 8000 y luego http://localhost:8000/src/pages/index.html).
+2. Los commits documentan el avance del desarrollo con mensajes claros y coherentes, verificables en la ronda de preguntas de la Entrega II.
+3. El repositorio documenta cómo ejecutar el proyecto localmente (npm install y luego npm run dev, en http://localhost:5173/).
 4. El proyecto comprimido que se entrega corresponde al mismo estado publicado en el repositorio público.
 5. Este documento declara la modalidad individual de desarrollo autorizada por el docente, de modo que el historial de un solo autor es verificable como tal.</t>
         </is>
       </c>
-      <c r="H23" s="12" t="inlineStr">
-        <is>
-          <t>Solicitado</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="319" customHeight="1">
-      <c r="A24" s="12" t="inlineStr">
+      <c r="H34" s="12" t="inlineStr">
+        <is>
+          <t>Solicitado</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="353" customHeight="1">
+      <c r="A35" s="12" t="inlineStr">
         <is>
           <t>RNF-08</t>
         </is>
       </c>
-      <c r="B24" s="12" t="inlineStr">
+      <c r="B35" s="12" t="inlineStr">
         <is>
           <t>Interfaces de usuario: menú superior, barra lateral, pie de página y panel administrativo</t>
         </is>
       </c>
-      <c r="C24" s="12" t="inlineStr">
+      <c r="C35" s="12" t="inlineStr">
         <is>
           <t>No Funcional</t>
         </is>
       </c>
-      <c r="D24" s="12" t="inlineStr">
+      <c r="D35" s="12" t="inlineStr">
         <is>
           <t>No funcional de producto</t>
         </is>
       </c>
-      <c r="E24" s="12" t="inlineStr">
+      <c r="E35" s="12" t="inlineStr">
         <is>
           <t>Cliente, Administrador logístico, Administrador</t>
         </is>
       </c>
-      <c r="F24" s="12" t="inlineStr">
-        <is>
-          <t>Las interfaces de usuario serán páginas web. Las vistas públicas son inicio, productos, detalle de producto, blogs, detalle de blog, nosotros, contacto, carrito, registro e inicio de sesión; las vistas administrativas son el home del panel, los mantenedores de Productos y de Usuarios, y el listado y detalle de órdenes.
-Toda vista pública presenta un menú superior de navegación con el logo de la tienda, los enlaces a Inicio, Productos, Blogs, Nosotros y Contacto y un acceso al carrito de compras que muestra la cantidad de ítems; un área de contenido central para la funcionalidad de cada vista; y un pie de página informativo con el nombre de la tienda, los enlaces de navegación principales, los datos de contacto de la empresa y el año. Las vistas de tienda presentan además una barra lateral con accesos a las categorías del catálogo. La página de inicio presenta, por sobre el listado de productos, un componente principal con la información y la imagen de la tienda, y bajo ese listado un video embebido que demuestra el asistente de armado. La vista "Nosotros" presenta la información institucional de la empresa y de sus desarrolladores (RF-15).
-El panel de administración utiliza un menú lateral vertical visible con los accesos a los mantenedores. El asistente de armado se presenta como un flujo guiado paso a paso, una categoría de componente a la vez, dentro del área de contenido. El diseño es responsivo y consistente en todas las páginas gracias a una hoja de estilos CSS externa y a los componentes de Bootstrap.</t>
-        </is>
-      </c>
-      <c r="G24" s="12" t="inlineStr">
-        <is>
-          <t>1. Toda vista pública muestra el menú superior con el logo de la tienda y los enlaces a Inicio, Productos, Blogs, Nosotros y Contacto, más el acceso al carrito de compras.
-2. La página de inicio presenta un componente principal con la información y la imagen de la tienda, visible antes del listado de productos.
-3. Toda vista de tienda muestra la barra lateral con los accesos a las categorías del catálogo.
+      <c r="F35" s="12" t="inlineStr">
+        <is>
+          <t>Las interfaces de usuario serán pantallas de la aplicación web, resueltas por rutas del cliente. Las vistas públicas son inicio, productos, categorías, ofertas, detalle de producto, armado de PC, carrito, pago, confirmación o rechazo del pago, blogs, detalle de blog, nosotros, contacto, registro, inicio de sesión, perfil, mis compras y detalle de compra; las vistas administrativas son el home del panel, los mantenedores de Productos, Categorías y Usuarios (con la ficha de cada usuario), los productos críticos, el listado y detalle de órdenes, los reportes y el perfil.
+Toda vista pública presenta un menú superior de navegación con el logo de la tienda, los enlaces a Inicio, Productos, Categorías, Ofertas, Armar mi PC, Blogs, Nosotros y Contacto, una caja de búsqueda y un acceso al carrito de compras que muestra la cantidad de ítems; un área de contenido central para la funcionalidad de cada vista; y un pie de página informativo con el nombre de la tienda, los enlaces de navegación principales, los datos de contacto de la empresa y el año. Las vistas de catálogo, ofertas, armado y carrito presentan además una barra lateral con accesos a las categorías del catálogo. La página de inicio presenta, por sobre el listado de productos, un componente principal con la información y la imagen de la tienda, y bajo ese listado un video embebido que demuestra el asistente de armado. La vista "Nosotros" presenta la información institucional de la empresa y de sus desarrolladores (RF-15).
+El panel de administración utiliza un menú lateral vertical visible con los accesos que corresponden al rol, y un home con indicadores. El asistente de armado se presenta como un flujo guiado paso a paso, una categoría de componente a la vez, dentro del área de contenido. El diseño es responsivo y consistente en todas las páginas gracias a una hoja de estilos CSS externa y a los componentes de Bootstrap.</t>
+        </is>
+      </c>
+      <c r="G35" s="12" t="inlineStr">
+        <is>
+          <t>1. Toda vista pública muestra el menú superior con el logo de la tienda y los enlaces a Inicio, Productos, Categorías, Ofertas, Armar mi PC, Blogs, Nosotros y Contacto, más la caja de búsqueda y el acceso al carrito de compras con su contador.
+2. En la página de inicio, el componente principal con la información y la imagen de la tienda aparece antes del listado de productos, y el video demostrativo del asistente, después.
+3. Las vistas de catálogo, ofertas, armado y carrito muestran la barra lateral con los accesos a las categorías del catálogo.
 4. Toda vista pública muestra un pie de página con el nombre de la tienda, los enlaces de navegación principales, los datos de contacto y el año.
-5. El home administrativo presenta un menú vertical visible cuyas opciones abren los mantenedores de Productos y Usuarios (RF-10 y RF-11).
+5. El home administrativo presenta indicadores (productos, críticos, usuarios y órdenes) y accesos a Productos, Críticos, Categorías, Usuarios, Órdenes y Reportes (RF-10, RF-11, RF-12, RF-25, RF-26 y RF-27).
 6. La vista "Nosotros" es accesible desde el menú superior de cualquier vista pública.</t>
         </is>
       </c>
-      <c r="H24" s="12" t="inlineStr">
+      <c r="H35" s="12" t="inlineStr">
+        <is>
+          <t>Solicitado</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="158" customHeight="1">
+      <c r="A36" s="12" t="inlineStr">
+        <is>
+          <t>RNF-09</t>
+        </is>
+      </c>
+      <c r="B36" s="12" t="inlineStr">
+        <is>
+          <t>Calidad y pruebas: pruebas unitarias con Vitest y Testing Library</t>
+        </is>
+      </c>
+      <c r="C36" s="12" t="inlineStr">
+        <is>
+          <t>No Funcional</t>
+        </is>
+      </c>
+      <c r="D36" s="12" t="inlineStr">
+        <is>
+          <t>No funcional de producto</t>
+        </is>
+      </c>
+      <c r="E36" s="12" t="inlineStr">
+        <is>
+          <t>Desarrollador, Docente evaluador</t>
+        </is>
+      </c>
+      <c r="F36" s="12" t="inlineStr">
+        <is>
+          <t>El comportamiento del sistema debe verificarse con pruebas unitarias automatizadas, escritas con Vitest y Testing Library, que cubran los componentes React (renderizado, renderizado condicional, props, estado y eventos), las reglas de negocio, la capa de datos, los hooks y los contextos, y que puedan ejecutarse en cualquier momento con un solo comando. El alcance, la estrategia y los resultados de las pruebas se documentan en docs/cobertura-testing.md.</t>
+        </is>
+      </c>
+      <c r="G36" s="12" t="inlineStr">
+        <is>
+          <t>1. Las pruebas unitarias se escriben con Vitest y Testing Library, junto al archivo que prueban, y npm run test:run las pasa todas.
+2. Cubren el renderizado, el renderizado condicional, las props, el estado y los eventos de los componentes, además de las reglas de src/logic/, src/utils/ y src/data/, los hooks y los contextos.
+3. Usan mocks (vi.fn, vi.spyOn y reloj simulado) para el almacenamiento, la consola y la fecha.
+4. npm run coverage genera el informe de cobertura v8; docs/cobertura-testing.md registra el alcance y los resultados (99,32 % de sentencias, 94,58 % de ramas, 99,80 % de funciones y 99,51 % de líneas, con 760 pruebas).</t>
+        </is>
+      </c>
+      <c r="H36" s="12" t="inlineStr">
         <is>
           <t>Solicitado</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H24"/>
+  <autoFilter ref="A1:H36"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>